<commit_message>
NAKO Fruits: now has the variable a_ui_f0401 Tracy DPEs: undertermined for varaibles which will be harmonised later.
</commit_message>
<xml_diff>
--- a/analyst/Franzi/rmonize/data_proc_elem/DPE_NAKO_FRANZI.xlsx
+++ b/analyst/Franzi/rmonize/data_proc_elem/DPE_NAKO_FRANZI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Franzi\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13952177-A59D-40DF-9458-5263F235724B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CE6FEBE-F65D-4B85-B661-900D07BBE46C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1698,21 +1698,18 @@
         <v>13</v>
       </c>
       <c r="E17" s="2"/>
-      <c r="F17" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>256</v>
+      <c r="G17" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
@@ -1725,18 +1722,21 @@
       <c r="D18" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7" t="s">
-        <v>273</v>
-      </c>
-      <c r="K18" s="7" t="s">
-        <v>273</v>
+      <c r="F18" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
@@ -3043,7 +3043,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="73" spans="2:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
         <v>154</v>
       </c>

</xml_diff>